<commit_message>
Completed Milestone 2 - Documentation
</commit_message>
<xml_diff>
--- a/project_documents/Defect Log.xlsx
+++ b/project_documents/Defect Log.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Desktop\LLM-Evaluation-system\project_documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A18EAABD-8483-4FDC-A46B-ADFB61E279BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{670B53EE-5AFA-4B20-A3B6-16E6E9FD5BF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{C21410EB-4A31-42C0-82E7-ACB6D7E14061}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="65">
   <si>
     <t>Description</t>
   </si>
@@ -171,6 +171,66 @@
   </si>
   <si>
     <t>FastAPI endpoint returned an import error</t>
+  </si>
+  <si>
+    <t>Sprint 2</t>
+  </si>
+  <si>
+    <t>AI Evaluation</t>
+  </si>
+  <si>
+    <t>Accuracy improved</t>
+  </si>
+  <si>
+    <t>Retrieval</t>
+  </si>
+  <si>
+    <t>Overall score fixed</t>
+  </si>
+  <si>
+    <t>Evaluation displayed correctly</t>
+  </si>
+  <si>
+    <t>Accuracy score was inconsistent</t>
+  </si>
+  <si>
+    <t>Improved prompt and scoring logic</t>
+  </si>
+  <si>
+    <t>Hallucination detection gave incorrect result</t>
+  </si>
+  <si>
+    <t>Updated hallucination prompt</t>
+  </si>
+  <si>
+    <t>Detection improved</t>
+  </si>
+  <si>
+    <t>Retrieved reference was not relevant</t>
+  </si>
+  <si>
+    <t>Improved retrieval logic</t>
+  </si>
+  <si>
+    <t>Judge Agent UI alignment issue</t>
+  </si>
+  <si>
+    <t>Updated dashboard layout</t>
+  </si>
+  <si>
+    <t>Dashboard improved</t>
+  </si>
+  <si>
+    <t>Overall score displayed incorrectly</t>
+  </si>
+  <si>
+    <t>Corrected score calculation</t>
+  </si>
+  <si>
+    <t>Evaluation response display issue</t>
+  </si>
+  <si>
+    <t>Fixed response display logic</t>
   </si>
 </sst>
 </file>
@@ -597,23 +657,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0509AE75-BD02-4198-8895-86DED6CA58B2}">
-  <dimension ref="A1:K9"/>
+  <dimension ref="A1:K15"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="8.1796875" customWidth="1"/>
     <col min="2" max="2" width="11.08984375" customWidth="1"/>
     <col min="3" max="3" width="12" customWidth="1"/>
-    <col min="4" max="4" width="27.36328125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="39.6328125" style="1" customWidth="1"/>
     <col min="5" max="5" width="11" customWidth="1"/>
     <col min="6" max="6" width="12.453125" customWidth="1"/>
     <col min="7" max="7" width="13.26953125" customWidth="1"/>
-    <col min="8" max="8" width="25.81640625" style="1" customWidth="1"/>
+    <col min="8" max="8" width="46.08984375" style="1" customWidth="1"/>
     <col min="9" max="9" width="12.26953125" customWidth="1"/>
     <col min="10" max="10" width="12.7265625" customWidth="1"/>
-    <col min="11" max="11" width="20.81640625" style="1" customWidth="1"/>
+    <col min="11" max="11" width="27.90625" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="26" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>8</v>
       </c>
@@ -648,7 +708,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="37.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3">
         <v>1</v>
       </c>
@@ -683,7 +743,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="25" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="3">
         <v>2</v>
       </c>
@@ -718,7 +778,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="37.5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="3">
         <v>3</v>
       </c>
@@ -753,7 +813,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="25" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="3">
         <v>4</v>
       </c>
@@ -788,7 +848,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="25" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="3">
         <v>5</v>
       </c>
@@ -823,7 +883,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="25" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="3">
         <v>6</v>
       </c>
@@ -858,7 +918,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="25" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="3">
         <v>7</v>
       </c>
@@ -893,7 +953,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="9" spans="1:11" ht="25" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="3">
         <v>8</v>
       </c>
@@ -926,6 +986,216 @@
       </c>
       <c r="K9" s="5" t="s">
         <v>41</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="3">
+        <v>9</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C10" s="4">
+        <v>46213</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G10" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="H10" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="I10" s="4">
+        <v>46213</v>
+      </c>
+      <c r="J10" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="K10" s="5" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="3">
+        <v>10</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C11" s="4">
+        <v>46214</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G11" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="H11" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="I11" s="4">
+        <v>46214</v>
+      </c>
+      <c r="J11" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="K11" s="5" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="3">
+        <v>11</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C12" s="4">
+        <v>46216</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G12" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="H12" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="I12" s="4">
+        <v>46216</v>
+      </c>
+      <c r="J12" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="K12" s="5" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="3">
+        <v>12</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C13" s="4">
+        <v>46218</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G13" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="H13" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="I13" s="4">
+        <v>46218</v>
+      </c>
+      <c r="J13" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="K13" s="5" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="3">
+        <v>13</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C14" s="4">
+        <v>46220</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G14" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="H14" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="I14" s="4">
+        <v>46220</v>
+      </c>
+      <c r="J14" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="K14" s="5" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="3">
+        <v>14</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C15" s="4">
+        <v>46222</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="F15" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G15" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="H15" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="I15" s="4">
+        <v>46222</v>
+      </c>
+      <c r="J15" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="K15" s="5" t="s">
+        <v>50</v>
       </c>
     </row>
   </sheetData>

</xml_diff>